<commit_message>
feat: ajustes de texto, remove emojis e atualiza template Excel
</commit_message>
<xml_diff>
--- a/assets/catalogo_kota_template.xlsx
+++ b/assets/catalogo_kota_template.xlsx
@@ -609,7 +609,7 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Válido até (AAAA-MM-DD)</t>
+          <t>Válido até (DD-MM-AAAA)</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>31-12-2025</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>Código interno do produto no seu sistema. Ex: CC2L, DET500</t>
+          <t>Código interno do produto. Ex: CC2L, DET500</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Data de validade do preço. Formato: AAAA-MM-DD. Ex: 2025-06-30</t>
+          <t>Data de validade do preço. Formato: DD-MM-AAAA. Ex: 31-12-2025</t>
         </is>
       </c>
     </row>

</xml_diff>